<commit_message>
fixing auto-fill EVB header information (order type & location)
</commit_message>
<xml_diff>
--- a/po_template/PO VH TEMPLATE.xlsx
+++ b/po_template/PO VH TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EVERBEST\NEW_GENERATOR\webapp\po_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191BB492-CF6E-4B49-B2D3-D0231DD58444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8EA150-129F-4FFD-ADF4-AD6F4F376941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2115" yWindow="2115" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1491,6 +1491,126 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1500,19 +1620,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1541,117 +1652,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3403,11 +3403,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="24.95" customHeight="1" thickBot="1">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="128" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="90"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="130"/>
       <c r="E1" s="1"/>
       <c r="F1" s="2"/>
       <c r="G1" s="3" t="s">
@@ -3421,10 +3421,10 @@
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="97" t="s">
+      <c r="B2" s="134" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="98"/>
+      <c r="C2" s="135"/>
       <c r="E2" s="7" t="s">
         <v>4</v>
       </c>
@@ -3437,8 +3437,8 @@
     </row>
     <row r="3" spans="1:16" ht="24.95" customHeight="1">
       <c r="A3" s="9"/>
-      <c r="B3" s="99"/>
-      <c r="C3" s="100"/>
+      <c r="B3" s="136"/>
+      <c r="C3" s="137"/>
       <c r="E3" s="10"/>
       <c r="G3" s="11" t="s">
         <v>6</v>
@@ -3451,10 +3451,10 @@
       <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="97" t="s">
+      <c r="B4" s="134" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="98"/>
+      <c r="C4" s="135"/>
       <c r="E4" s="10"/>
       <c r="G4" s="12" t="s">
         <v>8</v>
@@ -3467,10 +3467,10 @@
       <c r="A5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="101" t="s">
+      <c r="B5" s="138" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="102"/>
+      <c r="C5" s="139"/>
       <c r="E5" s="10"/>
       <c r="G5" s="12" t="s">
         <v>11</v>
@@ -3481,8 +3481,8 @@
     </row>
     <row r="6" spans="1:16" ht="24.95" customHeight="1" thickBot="1">
       <c r="A6" s="13"/>
-      <c r="B6" s="103"/>
-      <c r="C6" s="104"/>
+      <c r="B6" s="140"/>
+      <c r="C6" s="141"/>
       <c r="E6" s="14"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -3504,13 +3504,13 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:16" ht="30" customHeight="1">
-      <c r="A8" s="108" t="s">
+      <c r="A8" s="91" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="113" t="s">
+      <c r="B8" s="96" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="113" t="s">
+      <c r="C8" s="96" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="142" t="s">
@@ -3527,16 +3527,16 @@
       </c>
     </row>
     <row r="9" spans="1:16" ht="30" customHeight="1">
-      <c r="A9" s="109"/>
-      <c r="B9" s="114"/>
-      <c r="C9" s="114"/>
+      <c r="A9" s="92"/>
+      <c r="B9" s="97"/>
+      <c r="C9" s="97"/>
       <c r="D9" s="143"/>
       <c r="E9" s="146"/>
       <c r="F9" s="148"/>
       <c r="G9" s="150"/>
     </row>
     <row r="10" spans="1:16" ht="30" customHeight="1">
-      <c r="A10" s="110"/>
+      <c r="A10" s="93"/>
       <c r="B10" s="17" t="s">
         <v>19</v>
       </c>
@@ -3555,7 +3555,7 @@
       </c>
     </row>
     <row r="11" spans="1:16" ht="30" customHeight="1">
-      <c r="A11" s="111"/>
+      <c r="A11" s="94"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="22"/>
@@ -3569,7 +3569,7 @@
       </c>
     </row>
     <row r="12" spans="1:16" ht="30" customHeight="1">
-      <c r="A12" s="112"/>
+      <c r="A12" s="95"/>
       <c r="B12" s="26"/>
       <c r="C12" s="27"/>
       <c r="D12" s="28"/>
@@ -3694,10 +3694,10 @@
       <c r="A21" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="115" t="s">
+      <c r="B21" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="116"/>
+      <c r="C21" s="99"/>
       <c r="D21" s="42"/>
       <c r="E21" s="42"/>
       <c r="F21" s="42"/>
@@ -3705,8 +3705,8 @@
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1">
       <c r="A22" s="53"/>
-      <c r="B22" s="117"/>
-      <c r="C22" s="118"/>
+      <c r="B22" s="100"/>
+      <c r="C22" s="101"/>
       <c r="D22" s="42"/>
       <c r="E22" s="42"/>
       <c r="F22" s="42"/>
@@ -3754,144 +3754,144 @@
       <c r="H26" s="4"/>
     </row>
     <row r="27" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A27" s="128" t="s">
+      <c r="A27" s="111" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="129"/>
-      <c r="C27" s="129"/>
-      <c r="D27" s="129"/>
-      <c r="E27" s="129"/>
-      <c r="F27" s="129"/>
-      <c r="G27" s="129"/>
-      <c r="H27" s="130"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
+      <c r="F27" s="112"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="113"/>
     </row>
     <row r="28" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A28" s="131">
+      <c r="A28" s="114">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="B28" s="132"/>
-      <c r="C28" s="132"/>
-      <c r="D28" s="132"/>
-      <c r="E28" s="132"/>
-      <c r="F28" s="132"/>
-      <c r="G28" s="132"/>
-      <c r="H28" s="133"/>
+      <c r="B28" s="115"/>
+      <c r="C28" s="115"/>
+      <c r="D28" s="115"/>
+      <c r="E28" s="115"/>
+      <c r="F28" s="115"/>
+      <c r="G28" s="115"/>
+      <c r="H28" s="116"/>
     </row>
     <row r="29" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A29" s="131">
+      <c r="A29" s="114">
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="B29" s="132"/>
-      <c r="C29" s="132"/>
-      <c r="D29" s="132"/>
-      <c r="E29" s="132"/>
-      <c r="F29" s="132"/>
-      <c r="G29" s="132"/>
-      <c r="H29" s="133"/>
+      <c r="B29" s="115"/>
+      <c r="C29" s="115"/>
+      <c r="D29" s="115"/>
+      <c r="E29" s="115"/>
+      <c r="F29" s="115"/>
+      <c r="G29" s="115"/>
+      <c r="H29" s="116"/>
     </row>
     <row r="30" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A30" s="119"/>
-      <c r="B30" s="120"/>
-      <c r="C30" s="119"/>
-      <c r="D30" s="125"/>
-      <c r="E30" s="91"/>
-      <c r="F30" s="139"/>
-      <c r="G30" s="91"/>
-      <c r="H30" s="92"/>
+      <c r="A30" s="102"/>
+      <c r="B30" s="103"/>
+      <c r="C30" s="102"/>
+      <c r="D30" s="108"/>
+      <c r="E30" s="122"/>
+      <c r="F30" s="123"/>
+      <c r="G30" s="122"/>
+      <c r="H30" s="131"/>
     </row>
     <row r="31" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A31" s="121"/>
-      <c r="B31" s="122"/>
-      <c r="C31" s="121"/>
-      <c r="D31" s="126"/>
-      <c r="E31" s="93"/>
-      <c r="F31" s="140"/>
-      <c r="G31" s="93"/>
-      <c r="H31" s="94"/>
+      <c r="A31" s="104"/>
+      <c r="B31" s="105"/>
+      <c r="C31" s="104"/>
+      <c r="D31" s="109"/>
+      <c r="E31" s="124"/>
+      <c r="F31" s="125"/>
+      <c r="G31" s="124"/>
+      <c r="H31" s="132"/>
     </row>
     <row r="32" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A32" s="121"/>
-      <c r="B32" s="122"/>
-      <c r="C32" s="121"/>
-      <c r="D32" s="126"/>
-      <c r="E32" s="93"/>
-      <c r="F32" s="140"/>
-      <c r="G32" s="93"/>
-      <c r="H32" s="94"/>
+      <c r="A32" s="104"/>
+      <c r="B32" s="105"/>
+      <c r="C32" s="104"/>
+      <c r="D32" s="109"/>
+      <c r="E32" s="124"/>
+      <c r="F32" s="125"/>
+      <c r="G32" s="124"/>
+      <c r="H32" s="132"/>
     </row>
     <row r="33" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A33" s="121"/>
-      <c r="B33" s="122"/>
-      <c r="C33" s="121"/>
-      <c r="D33" s="126"/>
-      <c r="E33" s="93"/>
-      <c r="F33" s="140"/>
-      <c r="G33" s="93"/>
-      <c r="H33" s="94"/>
+      <c r="A33" s="104"/>
+      <c r="B33" s="105"/>
+      <c r="C33" s="104"/>
+      <c r="D33" s="109"/>
+      <c r="E33" s="124"/>
+      <c r="F33" s="125"/>
+      <c r="G33" s="124"/>
+      <c r="H33" s="132"/>
     </row>
     <row r="34" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A34" s="121"/>
-      <c r="B34" s="122"/>
-      <c r="C34" s="121"/>
-      <c r="D34" s="126"/>
-      <c r="E34" s="93"/>
-      <c r="F34" s="140"/>
-      <c r="G34" s="93"/>
-      <c r="H34" s="94"/>
+      <c r="A34" s="104"/>
+      <c r="B34" s="105"/>
+      <c r="C34" s="104"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="124"/>
+      <c r="F34" s="125"/>
+      <c r="G34" s="124"/>
+      <c r="H34" s="132"/>
     </row>
     <row r="35" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A35" s="121"/>
-      <c r="B35" s="122"/>
-      <c r="C35" s="121"/>
-      <c r="D35" s="126"/>
-      <c r="E35" s="93"/>
-      <c r="F35" s="140"/>
-      <c r="G35" s="93"/>
-      <c r="H35" s="94"/>
+      <c r="A35" s="104"/>
+      <c r="B35" s="105"/>
+      <c r="C35" s="104"/>
+      <c r="D35" s="109"/>
+      <c r="E35" s="124"/>
+      <c r="F35" s="125"/>
+      <c r="G35" s="124"/>
+      <c r="H35" s="132"/>
     </row>
     <row r="36" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A36" s="121"/>
-      <c r="B36" s="122"/>
-      <c r="C36" s="121"/>
-      <c r="D36" s="126"/>
-      <c r="E36" s="93"/>
-      <c r="F36" s="140"/>
-      <c r="G36" s="93"/>
-      <c r="H36" s="94"/>
+      <c r="A36" s="104"/>
+      <c r="B36" s="105"/>
+      <c r="C36" s="104"/>
+      <c r="D36" s="109"/>
+      <c r="E36" s="124"/>
+      <c r="F36" s="125"/>
+      <c r="G36" s="124"/>
+      <c r="H36" s="132"/>
     </row>
     <row r="37" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A37" s="123"/>
-      <c r="B37" s="124"/>
-      <c r="C37" s="123"/>
-      <c r="D37" s="127"/>
-      <c r="E37" s="95"/>
-      <c r="F37" s="141"/>
-      <c r="G37" s="95"/>
-      <c r="H37" s="96"/>
+      <c r="A37" s="106"/>
+      <c r="B37" s="107"/>
+      <c r="C37" s="106"/>
+      <c r="D37" s="110"/>
+      <c r="E37" s="126"/>
+      <c r="F37" s="127"/>
+      <c r="G37" s="126"/>
+      <c r="H37" s="133"/>
     </row>
     <row r="38" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A38" s="134">
+      <c r="A38" s="117">
         <f>D11</f>
         <v>0</v>
       </c>
-      <c r="B38" s="135"/>
-      <c r="C38" s="136">
+      <c r="B38" s="118"/>
+      <c r="C38" s="119">
         <f>D12</f>
         <v>0</v>
       </c>
-      <c r="D38" s="137"/>
-      <c r="E38" s="136">
+      <c r="D38" s="120"/>
+      <c r="E38" s="119">
         <f>D13</f>
         <v>0</v>
       </c>
-      <c r="F38" s="138"/>
-      <c r="G38" s="136">
+      <c r="F38" s="121"/>
+      <c r="G38" s="119">
         <f>D14</f>
         <v>0</v>
       </c>
-      <c r="H38" s="138"/>
+      <c r="H38" s="121"/>
     </row>
     <row r="39" spans="1:8" ht="24.95" customHeight="1">
       <c r="A39" s="64" t="s">
@@ -4047,11 +4047,11 @@
       <c r="H52" s="77"/>
     </row>
     <row r="53" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A53" s="105" t="s">
+      <c r="A53" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="B53" s="106"/>
-      <c r="C53" s="107"/>
+      <c r="B53" s="89"/>
+      <c r="C53" s="90"/>
       <c r="D53" s="84"/>
       <c r="E53" s="85"/>
       <c r="F53" s="84"/>
@@ -4060,6 +4060,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="G30:H37"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="B17:C18"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A12"/>
@@ -4076,19 +4089,6 @@
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="G38:H38"/>
     <mergeCell ref="E30:F37"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="G30:H37"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="B17:C18"/>
-    <mergeCell ref="F17:G17"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.11811023622047245" bottom="0.11811023622047245" header="0.11811023622047245" footer="0.11811023622047245"/>

</xml_diff>